<commit_message>
update fix driving range script from mac mini
</commit_message>
<xml_diff>
--- a/test_data/swing_ios_test_data.xlsx
+++ b/test_data/swing_ios_test_data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15340" activeTab="5"/>
+    <workbookView windowHeight="14600" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -21,8 +21,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Login!$A$4:$N$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Onboarding!$A$4:$Y$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Driving Range'!$A$4:$U$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tee Time'!$A$4:$U$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Players!$A$4:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tee Time'!$A$4:$U$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Players!$A$4:$O$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Swing Credits'!$A$4:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Event!$A$4:$S$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Add_ons!$A$4:$C$12</definedName>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="405">
   <si>
     <t>Swing iOS - Test Data</t>
   </si>
@@ -623,6 +623,9 @@
     <t>Verify Maximum Balls in One Booking</t>
   </si>
   <si>
+    <t>23 September 2026</t>
+  </si>
+  <si>
     <t>DR_014</t>
   </si>
   <si>
@@ -761,7 +764,7 @@
     <t>Booking Driving Range Without Promo Used Credit</t>
   </si>
   <si>
-    <t>23 September 2026</t>
+    <t>19:00</t>
   </si>
   <si>
     <t>Tee Time - Test Data</t>
@@ -815,9 +818,6 @@
     <t>Verify Explore Tee Time With Enable Swing Pass Partner</t>
   </si>
   <si>
-    <t>15 September 2026</t>
-  </si>
-  <si>
     <t>Day Session</t>
   </si>
   <si>
@@ -893,7 +893,7 @@
     <t>Book with Standard Tee Time, Host only, with auto applied promo</t>
   </si>
   <si>
-    <t>19 September 2026</t>
+    <t>24 September 2026</t>
   </si>
   <si>
     <t>TT_017</t>
@@ -902,7 +902,7 @@
     <t>Book with Standard Tee Time, Host  and invite player , with auto applied promo</t>
   </si>
   <si>
-    <t>20 September 2026</t>
+    <t>25 September 2026</t>
   </si>
   <si>
     <t>TT_018</t>
@@ -911,9 +911,6 @@
     <t>Book with Standard Tee Time, Host only, without promo</t>
   </si>
   <si>
-    <t>19 September 2027</t>
-  </si>
-  <si>
     <t>Night Session</t>
   </si>
   <si>
@@ -926,18 +923,12 @@
     <t>Book with Standard Tee Time, Host  and invite player , without promo</t>
   </si>
   <si>
-    <t>20 September 2027</t>
-  </si>
-  <si>
     <t>TT_020</t>
   </si>
   <si>
     <t>Book with Standard Tee Time, Host only, with apply redeemed promo</t>
   </si>
   <si>
-    <t>19 September 2028</t>
-  </si>
-  <si>
     <t>Standard Booking</t>
   </si>
   <si>
@@ -953,9 +944,6 @@
     <t>Book with Standard Tee Time, Host  and invite player , with apply redeemed promo</t>
   </si>
   <si>
-    <t>20 September 2028</t>
-  </si>
-  <si>
     <t>13:30 - 14:00</t>
   </si>
   <si>
@@ -963,9 +951,6 @@
   </si>
   <si>
     <t>Book with Standard Tee Time, Host only, with auto applied promo, with used credit</t>
-  </si>
-  <si>
-    <t>19 September 2029</t>
   </si>
   <si>
     <t>10:30 - 11:00</t>
@@ -4390,7 +4375,7 @@
         <v>170</v>
       </c>
       <c r="N17" s="21" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="O17" s="21" t="s">
         <v>185</v>
@@ -4413,10 +4398,10 @@
     </row>
     <row r="18" ht="34" spans="1:21">
       <c r="A18" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>158</v>
@@ -4452,7 +4437,7 @@
         <v>170</v>
       </c>
       <c r="N18" s="21" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="O18" s="21" t="s">
         <v>185</v>
@@ -4473,15 +4458,15 @@
         <v>47</v>
       </c>
       <c r="U18" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" customFormat="1" ht="34" spans="1:21">
       <c r="A19" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>158</v>
@@ -4532,21 +4517,21 @@
         <v>121</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="T19" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U19" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" customFormat="1" ht="34" spans="1:21">
       <c r="A20" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>158</v>
@@ -4597,21 +4582,21 @@
         <v>121</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="T20" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U20" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" ht="34" spans="1:21">
       <c r="A21" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>158</v>
@@ -4662,30 +4647,30 @@
         <v>121</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="T21" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U21" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" ht="34" spans="1:21">
       <c r="A22" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>74</v>
@@ -4733,24 +4718,24 @@
         <v>47</v>
       </c>
       <c r="U22" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" customFormat="1" ht="34" spans="1:21">
       <c r="A23" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>74</v>
@@ -4780,10 +4765,10 @@
         <v>184</v>
       </c>
       <c r="O23" s="21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P23" s="21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q23" s="4" t="s">
         <v>133</v>
@@ -4792,30 +4777,30 @@
         <v>121</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="T23" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U23" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" customFormat="1" ht="34" spans="1:21">
       <c r="A24" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>74</v>
@@ -4845,10 +4830,10 @@
         <v>184</v>
       </c>
       <c r="O24" s="21" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P24" s="21" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Q24" s="4" t="s">
         <v>133</v>
@@ -4857,30 +4842,30 @@
         <v>121</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="T24" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U24" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" ht="34" spans="1:21">
       <c r="A25" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>74</v>
@@ -4910,10 +4895,10 @@
         <v>184</v>
       </c>
       <c r="O25" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P25" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q25" s="4" t="s">
         <v>133</v>
@@ -4922,27 +4907,27 @@
         <v>121</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="T25" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U25" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" ht="34" spans="1:21">
       <c r="A26" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>65</v>
@@ -4972,13 +4957,13 @@
         <v>170</v>
       </c>
       <c r="N26" s="21" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="O26" s="21" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="P26" s="21" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="Q26" s="4" t="s">
         <v>133</v>
@@ -4987,27 +4972,27 @@
         <v>121</v>
       </c>
       <c r="S26" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="T26" s="4" t="s">
         <v>47</v>
       </c>
       <c r="U26" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="27" ht="34" spans="1:21">
       <c r="A27" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>65</v>
@@ -5040,10 +5025,10 @@
         <v>184</v>
       </c>
       <c r="O27" s="21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="P27" s="21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q27" s="4" t="s">
         <v>133</v>
@@ -5052,27 +5037,27 @@
         <v>121</v>
       </c>
       <c r="S27" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="T27" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="U27" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" ht="17" spans="1:21">
       <c r="A28" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>65</v>
@@ -5096,19 +5081,19 @@
         <v>162</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N28" s="23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O28" s="21" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="P28" s="21" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q28" s="4" t="s">
         <v>133</v>
@@ -5119,21 +5104,21 @@
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
       <c r="U28" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" ht="34" spans="1:21">
       <c r="A29" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>65</v>
@@ -5151,55 +5136,55 @@
         <v>47</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K29" s="4" t="s">
         <v>162</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N29" s="23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O29" s="21" t="s">
         <v>185</v>
       </c>
       <c r="P29" s="21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q29" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R29" s="21" t="s">
         <v>121</v>
       </c>
       <c r="S29" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="T29" s="4"/>
       <c r="U29" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="30" ht="34" spans="1:21">
       <c r="A30" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>158</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>74</v>
@@ -5214,7 +5199,7 @@
         <v>47</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>162</v>
@@ -5226,13 +5211,13 @@
         <v>170</v>
       </c>
       <c r="N30" s="21" t="s">
-        <v>238</v>
+        <v>192</v>
       </c>
       <c r="O30" s="21" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="P30" s="21" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="Q30" s="4" t="s">
         <v>133</v>
@@ -5247,7 +5232,7 @@
         <v>47</v>
       </c>
       <c r="U30" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -5293,7 +5278,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5321,12 +5306,12 @@
   <sheetData>
     <row r="1" ht="20.4" spans="1:21">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" ht="34" spans="1:21">
@@ -5358,7 +5343,7 @@
         <v>60</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>145</v>
@@ -5367,22 +5352,22 @@
         <v>146</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>148</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="S4" s="3" t="s">
         <v>155</v>
@@ -5396,10 +5381,10 @@
     </row>
     <row r="5" ht="34" spans="1:21">
       <c r="A5" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>20</v>
@@ -5429,10 +5414,10 @@
         <v>159</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
@@ -5449,10 +5434,10 @@
     </row>
     <row r="6" ht="34" spans="1:21">
       <c r="A6" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>20</v>
@@ -5482,10 +5467,10 @@
         <v>162</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -5502,10 +5487,10 @@
     </row>
     <row r="7" ht="34" spans="1:21">
       <c r="A7" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>20</v>
@@ -5535,10 +5520,10 @@
         <v>165</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
@@ -5555,10 +5540,10 @@
     </row>
     <row r="8" ht="34" spans="1:21">
       <c r="A8" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>20</v>
@@ -5588,13 +5573,13 @@
         <v>162</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N8" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>257</v>
@@ -5609,7 +5594,7 @@
         <v>121</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T8" s="4" t="s">
         <v>47</v>
@@ -5653,13 +5638,13 @@
         <v>162</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N9" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O9" s="4" t="s">
         <v>257</v>
@@ -5674,7 +5659,7 @@
         <v>121</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T9" s="4" t="s">
         <v>47</v>
@@ -5718,13 +5703,13 @@
         <v>162</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N10" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O10" s="4" t="s">
         <v>257</v>
@@ -5739,7 +5724,7 @@
         <v>121</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T10" s="4" t="s">
         <v>47</v>
@@ -5783,13 +5768,13 @@
         <v>162</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N11" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>257</v>
@@ -5804,7 +5789,7 @@
         <v>121</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T11" s="4" t="s">
         <v>47</v>
@@ -5848,13 +5833,13 @@
         <v>165</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N12" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O12" s="4" t="s">
         <v>257</v>
@@ -5869,7 +5854,7 @@
         <v>121</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T12" s="4"/>
       <c r="U12" s="4" t="s">
@@ -5911,13 +5896,13 @@
         <v>159</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N13" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O13" s="4" t="s">
         <v>257</v>
@@ -5932,7 +5917,7 @@
         <v>121</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T13" s="4"/>
       <c r="U13" s="4" t="s">
@@ -5953,7 +5938,7 @@
         <v>64</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>74</v>
@@ -5974,13 +5959,13 @@
         <v>162</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N14" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N14" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O14" s="4" t="s">
         <v>257</v>
@@ -5995,7 +5980,7 @@
         <v>121</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T14" s="4"/>
       <c r="U14" s="4" t="s">
@@ -6016,7 +6001,7 @@
         <v>64</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>74</v>
@@ -6037,13 +6022,13 @@
         <v>162</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N15" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N15" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O15" s="4" t="s">
         <v>257</v>
@@ -6058,7 +6043,7 @@
         <v>189</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T15" s="4"/>
       <c r="U15" s="4" t="s">
@@ -6079,7 +6064,7 @@
         <v>64</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>74</v>
@@ -6100,13 +6085,13 @@
         <v>162</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N16" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O16" s="4" t="s">
         <v>257</v>
@@ -6121,7 +6106,7 @@
         <v>189</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T16" s="4"/>
       <c r="U16" s="4" t="s">
@@ -6163,13 +6148,13 @@
         <v>162</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N17" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N17" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O17" s="4" t="s">
         <v>257</v>
@@ -6184,7 +6169,7 @@
         <v>121</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T17" s="4" t="s">
         <v>274</v>
@@ -6228,13 +6213,13 @@
         <v>165</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N18" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N18" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O18" s="4" t="s">
         <v>257</v>
@@ -6249,7 +6234,7 @@
         <v>189</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T18" s="4" t="s">
         <v>277</v>
@@ -6293,13 +6278,13 @@
         <v>159</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="N19" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
+      </c>
+      <c r="N19" s="21" t="s">
+        <v>192</v>
       </c>
       <c r="O19" s="4" t="s">
         <v>257</v>
@@ -6314,7 +6299,7 @@
         <v>121</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T19" s="4" t="s">
         <v>277</v>
@@ -6332,10 +6317,10 @@
         <v>20</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>74</v>
@@ -6356,10 +6341,10 @@
         <v>162</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N20" s="21" t="s">
         <v>282</v>
@@ -6377,7 +6362,7 @@
         <v>121</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T20" s="4" t="s">
         <v>274</v>
@@ -6395,10 +6380,10 @@
         <v>20</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>74</v>
@@ -6419,10 +6404,10 @@
         <v>162</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N21" s="21" t="s">
         <v>285</v>
@@ -6440,7 +6425,7 @@
         <v>186</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T21" s="4" t="s">
         <v>274</v>
@@ -6460,10 +6445,10 @@
         <v>20</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>74</v>
@@ -6484,19 +6469,19 @@
         <v>162</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N22" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="O22" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="O22" s="4" t="s">
+      <c r="P22" s="21" t="s">
         <v>289</v>
-      </c>
-      <c r="P22" s="21" t="s">
-        <v>290</v>
       </c>
       <c r="Q22" s="4" t="s">
         <v>259</v>
@@ -6505,7 +6490,7 @@
         <v>121</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T22" s="4"/>
       <c r="U22" s="4" t="s">
@@ -6514,19 +6499,19 @@
     </row>
     <row r="23" customFormat="1" ht="34" spans="1:21">
       <c r="A23" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>291</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>292</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>74</v>
@@ -6547,19 +6532,19 @@
         <v>162</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N23" s="21" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="O23" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="P23" s="21" t="s">
         <v>289</v>
-      </c>
-      <c r="P23" s="21" t="s">
-        <v>290</v>
       </c>
       <c r="Q23" s="4" t="s">
         <v>259</v>
@@ -6568,7 +6553,7 @@
         <v>186</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T23" s="4"/>
       <c r="U23" s="4" t="s">
@@ -6577,19 +6562,19 @@
     </row>
     <row r="24" customFormat="1" ht="34" spans="1:21">
       <c r="A24" s="4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>74</v>
@@ -6610,51 +6595,51 @@
         <v>162</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N24" s="21" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="O24" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="P24" s="21" t="s">
         <v>289</v>
       </c>
-      <c r="P24" s="21" t="s">
-        <v>290</v>
-      </c>
       <c r="Q24" s="4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="R24" s="21" t="s">
         <v>121</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="T24" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="U24" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" customFormat="1" ht="34" spans="1:21">
       <c r="A25" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>74</v>
@@ -6675,51 +6660,51 @@
         <v>162</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M25" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N25" s="21" t="s">
-        <v>302</v>
+        <v>192</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P25" s="21" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="Q25" s="4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="R25" s="21" t="s">
         <v>189</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="T25" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="U25" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" ht="34" spans="1:21">
       <c r="A26" s="4" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>74</v>
@@ -6734,25 +6719,25 @@
         <v>47</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K26" s="4" t="s">
         <v>162</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N26" s="21" t="s">
-        <v>306</v>
+        <v>282</v>
       </c>
       <c r="O26" s="4" t="s">
         <v>257</v>
       </c>
       <c r="P26" s="21" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="Q26" s="4" t="s">
         <v>259</v>
@@ -6761,22 +6746,25 @@
         <v>121</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="T26" s="4" t="s">
         <v>274</v>
       </c>
       <c r="U26" s="4"/>
     </row>
+    <row r="27" spans="1:21">
+      <c r="N27" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:U25" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:U26" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="D26 D5:D12 D13:D19 D20:D25">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D26">
       <formula1>"UI,Positive,Negative,E2E"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E26 E5:E25">
+    <dataValidation type="list" allowBlank="1" sqref="E5:E26">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6809,12 +6797,12 @@
   <sheetData>
     <row r="1" ht="20.4" spans="1:15">
       <c r="A1" s="1" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="2" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" ht="17" spans="1:15">
@@ -6822,13 +6810,13 @@
         <v>27</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>146</v>
@@ -6855,10 +6843,10 @@
         <v>154</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>7</v>
@@ -6872,16 +6860,16 @@
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>47</v>
@@ -6913,16 +6901,16 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
+        <v>310</v>
+      </c>
+      <c r="D6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F6" t="s">
         <v>315</v>
-      </c>
-      <c r="D6" t="s">
-        <v>319</v>
-      </c>
-      <c r="E6" t="s">
-        <v>319</v>
-      </c>
-      <c r="F6" t="s">
-        <v>320</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>47</v>
@@ -6954,28 +6942,28 @@
         <v>3</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>321</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>326</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>277</v>
@@ -6989,86 +6977,86 @@
     </row>
     <row r="8" ht="34" spans="1:15">
       <c r="A8" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
+        <v>310</v>
+      </c>
+      <c r="D8" t="s">
+        <v>314</v>
+      </c>
+      <c r="E8" t="s">
+        <v>314</v>
+      </c>
+      <c r="F8" t="s">
         <v>315</v>
       </c>
-      <c r="D8" t="s">
-        <v>319</v>
-      </c>
-      <c r="E8" t="s">
-        <v>319</v>
-      </c>
-      <c r="F8" t="s">
-        <v>320</v>
-      </c>
       <c r="K8" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" ht="34" spans="1:15">
       <c r="A9" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" t="s">
+        <v>316</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J9" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>326</v>
-      </c>
       <c r="K9" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" ht="17" spans="1:15">
       <c r="A10" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B10" s="4">
         <v>1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>47</v>
@@ -7092,22 +7080,22 @@
     </row>
     <row r="11" ht="17" spans="1:15">
       <c r="A11" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B11" s="4">
         <v>2</v>
       </c>
       <c r="C11" t="s">
+        <v>310</v>
+      </c>
+      <c r="D11" t="s">
+        <v>314</v>
+      </c>
+      <c r="E11" t="s">
+        <v>314</v>
+      </c>
+      <c r="F11" t="s">
         <v>315</v>
-      </c>
-      <c r="D11" t="s">
-        <v>319</v>
-      </c>
-      <c r="E11" t="s">
-        <v>319</v>
-      </c>
-      <c r="F11" t="s">
-        <v>320</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>47</v>
@@ -7131,34 +7119,34 @@
     </row>
     <row r="12" ht="17" spans="1:15">
       <c r="A12" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B12" s="4">
         <v>3</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J12" s="4" t="s">
         <v>321</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>326</v>
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4" t="s">
@@ -7169,7 +7157,7 @@
       <c r="O12" s="4"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:O9" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:O12" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <dataValidations count="1">
@@ -7203,12 +7191,12 @@
   <sheetData>
     <row r="1" ht="20.4" customHeight="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:11">
@@ -7231,10 +7219,10 @@
         <v>33</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>37</v>
@@ -7248,10 +7236,10 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="6" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>16</v>
@@ -7263,7 +7251,7 @@
         <v>65</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>47</v>
@@ -7272,10 +7260,10 @@
         <v>47</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>69</v>
@@ -7283,10 +7271,10 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="9" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>16</v>
@@ -7298,19 +7286,19 @@
         <v>73</v>
       </c>
       <c r="F6" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>338</v>
-      </c>
       <c r="J6" s="10" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>69</v>
@@ -7318,10 +7306,10 @@
     </row>
     <row r="7" ht="29" customHeight="1" spans="1:11">
       <c r="A7" s="6" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>16</v>
@@ -7333,19 +7321,19 @@
         <v>65</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="H7" s="8">
         <v>7500</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>69</v>
@@ -7353,10 +7341,10 @@
     </row>
     <row r="8" ht="29" customHeight="1" spans="1:11">
       <c r="A8" s="9" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>16</v>
@@ -7368,19 +7356,19 @@
         <v>65</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="H8" s="8">
         <v>750</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>69</v>
@@ -7435,12 +7423,12 @@
   <sheetData>
     <row r="1" ht="20.4" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="2" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:19">
@@ -7463,31 +7451,31 @@
         <v>33</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>106</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="P4" s="5" t="s">
         <v>155</v>
@@ -7496,7 +7484,7 @@
         <v>37</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="S4" s="5" t="s">
         <v>41</v>
@@ -7504,10 +7492,10 @@
     </row>
     <row r="5" ht="29" customHeight="1" spans="1:19">
       <c r="A5" s="6" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>24</v>
@@ -7519,7 +7507,7 @@
         <v>65</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>47</v>
@@ -7552,10 +7540,10 @@
         <v>47</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S5" s="7" t="s">
         <v>69</v>
@@ -7563,10 +7551,10 @@
     </row>
     <row r="6" ht="29" customHeight="1" spans="1:19">
       <c r="A6" s="9" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>24</v>
@@ -7578,10 +7566,10 @@
         <v>65</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>47</v>
@@ -7611,10 +7599,10 @@
         <v>47</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="R6" s="10" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S6" s="10" t="s">
         <v>69</v>
@@ -7622,10 +7610,10 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="6" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>24</v>
@@ -7637,13 +7625,13 @@
         <v>65</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>47</v>
@@ -7655,25 +7643,25 @@
         <v>123</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="O7" s="8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S7" s="7" t="s">
         <v>69</v>
@@ -7681,10 +7669,10 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="9" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>24</v>
@@ -7696,13 +7684,13 @@
         <v>65</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>47</v>
@@ -7714,25 +7702,25 @@
         <v>123</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="N8" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="O8" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="O8" s="8" t="s">
-        <v>378</v>
-      </c>
       <c r="P8" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S8" s="10" t="s">
         <v>69</v>
@@ -7740,10 +7728,10 @@
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="6" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>24</v>
@@ -7755,43 +7743,43 @@
         <v>65</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>123</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S9" s="7" t="s">
         <v>69</v>
@@ -7799,10 +7787,10 @@
     </row>
     <row r="10" spans="1:19">
       <c r="A10" s="9" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>24</v>
@@ -7814,13 +7802,13 @@
         <v>65</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>47</v>
@@ -7841,16 +7829,16 @@
         <v>47</v>
       </c>
       <c r="O10" s="8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="P10" s="8" t="s">
         <v>47</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>69</v>
@@ -7858,10 +7846,10 @@
     </row>
     <row r="11" spans="1:19">
       <c r="A11" s="6" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>24</v>
@@ -7873,13 +7861,13 @@
         <v>73</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>47</v>
@@ -7891,25 +7879,25 @@
         <v>123</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S11" s="7" t="s">
         <v>69</v>
@@ -7917,10 +7905,10 @@
     </row>
     <row r="12" ht="29" customHeight="1" spans="1:19">
       <c r="A12" s="9" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>24</v>
@@ -7932,13 +7920,13 @@
         <v>73</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>47</v>
@@ -7959,16 +7947,16 @@
         <v>47</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="P12" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>69</v>
@@ -8007,12 +7995,12 @@
   <sheetData>
     <row r="1" ht="20.4" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" ht="34" spans="1:3">
@@ -8020,18 +8008,18 @@
         <v>27</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" ht="17" spans="1:3">
       <c r="A5" s="4" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C5" s="4">
         <v>1</v>
@@ -8039,10 +8027,10 @@
     </row>
     <row r="6" ht="17" spans="1:3">
       <c r="A6" s="4" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="C6" s="4">
         <v>1</v>
@@ -8050,10 +8038,10 @@
     </row>
     <row r="7" ht="17" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="C7" s="4">
         <v>5</v>
@@ -8061,10 +8049,10 @@
     </row>
     <row r="8" ht="17" spans="1:3">
       <c r="A8" s="4" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C8" s="4">
         <v>1</v>
@@ -8075,7 +8063,7 @@
         <v>283</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="C9" s="4">
         <v>2</v>
@@ -8086,7 +8074,7 @@
         <v>283</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="C10" s="4">
         <v>1</v>
@@ -8097,7 +8085,7 @@
         <v>190</v>
       </c>
       <c r="B11" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C11">
         <v>20</v>
@@ -8105,10 +8093,10 @@
     </row>
     <row r="12" ht="17" spans="1:3">
       <c r="A12" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B12" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="C12">
         <v>1</v>

</xml_diff>